<commit_message>
keep: the filter database where the AutoFilter stays as Excel moves it, two known differences gone; Excel for Mac opened the two files again
writeKept now writes for filter-move-over and filter-move-end-down what Excel did
(the keep fix of the filter database). The Mac's struct-open ran again for the two
changed files; their prediction, what writeKept writes, was set after that run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/keep/struct-open/filter-move-end-down.xlsx
+++ b/test/excel/keep/struct-open/filter-move-end-down.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Library/Containers/com.microsoft.Excel/Data/tmp/fkeep-68964/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Library/Containers/com.microsoft.Excel/Data/tmp/fkeep-60236/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA112938-19CA-2C4F-B3E1-3BD0113A01AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1131C031-58C3-2044-A1C4-7FC8536F624C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Plain" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$C$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$C$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>